<commit_message>
v1.4.1 - Added documentations, screenshots, bugs and a CHANGELOG.md
</commit_message>
<xml_diff>
--- a/hardware/BOM.xlsx
+++ b/hardware/BOM.xlsx
@@ -1,19 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\baldu\Documents\Arduino\BalduHandbrake\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9448C4BE-B867-45D7-A78D-751908D7ADDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D362D9-58DB-49F3-AE29-6831FEC184F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{8A0C3255-D7A5-4095-B8D9-DD99EA93DA22}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{8A0C3255-D7A5-4095-B8D9-DD99EA93DA22}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="ADS1115" sheetId="1" r:id="rId1"/>
+    <sheet name="ADS122C04" sheetId="2" r:id="rId2"/>
+    <sheet name="ADS122C04-Load Cell" sheetId="3" r:id="rId3"/>
+    <sheet name="NAU7802" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="27">
   <si>
     <t>Momentary Button</t>
   </si>
@@ -50,18 +53,12 @@
     <t>ADS1115 Module</t>
   </si>
   <si>
-    <t>Wavesahre ESP3-S3 Zero</t>
-  </si>
-  <si>
     <t>1/8 NPT 5V 500psi/1000psi Pressure Transducer</t>
   </si>
   <si>
     <t>Logic Voltage Converter</t>
   </si>
   <si>
-    <t>220R Resistor</t>
-  </si>
-  <si>
     <t>104 Capacitor</t>
   </si>
   <si>
@@ -75,16 +72,81 @@
   </si>
   <si>
     <t>KY-040 Rotary Encoder</t>
+  </si>
+  <si>
+    <t>Waveshare ESP3-S3 Zero</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/gp/product/B0CRQXGMWD/ref=ox_sc_act_title_3?th=1</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/HiLetgo-Converter-Programmable-Amplifier-Development/dp/B01DLHKMO2</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/SparkFun-12009-Logic-Converter-Bi-Directional/dp/B088FYQJYZ/ref=sr_1_4</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/1-5inch-RGB-OLED-Module-Interface/dp/B07V579YK2/ref=sr_1_1</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/waveshare-Mini-Development-Board-ESP32-S3FH4R2/dp/B0CS6VS1DJ/ref=sr_1_2</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/uxcell-Momentary-Button-Switch-Mounting/dp/B0D5L7H9D2/ref=sr_1_4</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/KY-040-Degrees-Encoder-15%C3%9716-5mm-Potentiometer/dp/B09LVG8ZGR/ref=sr_1_4</t>
+  </si>
+  <si>
+    <t>107 Capacitor</t>
+  </si>
+  <si>
+    <t>4.7k Ohm Resistor</t>
+  </si>
+  <si>
+    <t>220 Ohm Resistor</t>
+  </si>
+  <si>
+    <t>https://www.adafruit.com/product/6432</t>
+  </si>
+  <si>
+    <t>ADS122C04 Module</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/Single-Mechanic-Electronic-Switch-Weight/dp/B088GY1HFL/ref=sr_1_7</t>
+  </si>
+  <si>
+    <t>NA151 Single Point Load Cell Mechanic to Electronic Switch Weight Sensor (200kg)</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/Acquisition-Electronic-Collection-Biomedical-Automation/dp/B0GXJB7GX5/ref=sr_1_3</t>
+  </si>
+  <si>
+    <t>NAU7802 Module</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -107,13 +169,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -446,92 +511,569 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EC3CCF4-976C-4F01-AB6D-8B26631F54D3}">
-  <dimension ref="B6:C16"/>
+  <dimension ref="B6:D18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="39.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="102.6328125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
         <v>10</v>
       </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D8" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D9" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D11" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D12" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D8" r:id="rId1" xr:uid="{2AC574D1-E75C-4C16-8793-5DC1F00D2E7A}"/>
+    <hyperlink ref="D9" r:id="rId2" xr:uid="{A49ABE40-8C09-46B8-A7C4-237D03907574}"/>
+    <hyperlink ref="D10" r:id="rId3" xr:uid="{52533811-AB3F-44C2-BA63-D7079413FC94}"/>
+    <hyperlink ref="D11" r:id="rId4" xr:uid="{C77DF809-3B0D-428E-8ABA-39283E568489}"/>
+    <hyperlink ref="D7" r:id="rId5" xr:uid="{543E5E2F-4822-4CCA-9520-4F6EA0C57BF5}"/>
+    <hyperlink ref="D12" r:id="rId6" xr:uid="{4AD780B7-4FF1-4894-BD09-E736B0619C13}"/>
+    <hyperlink ref="D13" r:id="rId7" xr:uid="{67DAE12B-D8E2-4097-85DD-8FEB4749EB07}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46232997-CC8F-452F-BBAE-F3FB5883251B}">
+  <dimension ref="B6:D18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="39.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="102.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>0</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D8" r:id="rId1" xr:uid="{072CD122-A933-465B-8DF5-7B53E6DF2962}"/>
+    <hyperlink ref="D10" r:id="rId2" xr:uid="{3D27CC2F-762A-42DC-8BBF-A26EDE1315DA}"/>
+    <hyperlink ref="D11" r:id="rId3" xr:uid="{3D9D461A-DC44-4688-BC10-D07054BBDB87}"/>
+    <hyperlink ref="D7" r:id="rId4" xr:uid="{7F829B6D-20C8-4F0E-9548-A26B7137CD37}"/>
+    <hyperlink ref="D12" r:id="rId5" xr:uid="{85573672-ADE8-411E-90E0-3BA323609530}"/>
+    <hyperlink ref="D13" r:id="rId6" xr:uid="{17777557-62BD-43E2-AA66-2EF6DBB22591}"/>
+    <hyperlink ref="D9" r:id="rId7" xr:uid="{22BC4919-6780-43FF-892B-B04D4CF9F2A5}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1600F3C5-807B-489A-A43C-AB9CF6F5F683}">
+  <dimension ref="B6:D17"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="39.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="102.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B15">
+        <v>4</v>
+      </c>
       <c r="C15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D10" r:id="rId1" xr:uid="{E16F87E5-CBAE-41CB-9835-FC2E544B3D5C}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{2C0BAA52-EA7A-4BE9-B406-AC5696F9A473}"/>
+    <hyperlink ref="D11" r:id="rId3" xr:uid="{18ACE3A2-D87E-43A7-A997-921C1ABEFED0}"/>
+    <hyperlink ref="D12" r:id="rId4" xr:uid="{AEB14E19-5057-4556-B266-5AE81176BEBA}"/>
+    <hyperlink ref="D9" r:id="rId5" xr:uid="{3949099C-EDE3-4727-9A04-F6B078E67A56}"/>
+    <hyperlink ref="D8" r:id="rId6" xr:uid="{4075108B-146C-459A-A84B-BFC993800EFB}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3010EDDE-8ED7-4807-9CE7-FB26622845C8}">
+  <dimension ref="B6:D17"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="39.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="102.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B15">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B16">
+        <v>3</v>
+      </c>
       <c r="C16" t="s">
-        <v>8</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D10" r:id="rId1" xr:uid="{26026B96-1A2F-4306-8BDE-B116C6567933}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{BF3CF66D-2F7E-431C-80FE-C65FD8D944DD}"/>
+    <hyperlink ref="D11" r:id="rId3" xr:uid="{0B623AC0-1435-454B-B291-A0C1634380AA}"/>
+    <hyperlink ref="D12" r:id="rId4" xr:uid="{F28F9899-6C57-45B0-BD78-FBE5543E5363}"/>
+    <hyperlink ref="D8" r:id="rId5" xr:uid="{69FB3612-34AB-4850-B211-6322610A7F01}"/>
+    <hyperlink ref="D9" r:id="rId6" xr:uid="{E4F0878E-F4D2-435D-B0D6-D866409DE62D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>